<commit_message>
Added CarLoanTestData excel file
</commit_message>
<xml_diff>
--- a/test-data/CarLoanTestData.xlsx
+++ b/test-data/CarLoanTestData.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\2478620\Downloads\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{F96608D4-8CFD-4AF1-8C84-6F9C4D9AA24D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{35ED5EFB-BEF0-4E53-BF41-3380EE97985B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="12220" xr2:uid="{1CC61DC1-D1E0-4F49-928F-2DBB17E33D24}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="12220" xr2:uid="{C06392C3-B2F8-4A4B-BB2F-76D7B47CBD86}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -38,34 +38,34 @@
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
 <sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="10" uniqueCount="10">
   <si>
-    <t>LoanAmount</t>
-  </si>
-  <si>
-    <t>InterestRate</t>
+    <t>Loan Amount</t>
+  </si>
+  <si>
+    <t>Interest Rate</t>
   </si>
   <si>
     <t>Tenure</t>
   </si>
   <si>
+    <t>Expected Amount</t>
+  </si>
+  <si>
+    <t>Actual Amount</t>
+  </si>
+  <si>
+    <t>Status</t>
+  </si>
+  <si>
     <t>TestCaseName</t>
   </si>
   <si>
-    <t>Expected EMI</t>
-  </si>
-  <si>
-    <t>Actual EMI</t>
-  </si>
-  <si>
-    <t>Status</t>
-  </si>
-  <si>
     <t>Car_15L_9.5_1yr</t>
   </si>
   <si>
-    <t>Car_20L_8.5_2yr</t>
-  </si>
-  <si>
-    <t>Car_50L_10_5yr</t>
+    <t>Car_20L_8.5_1yr</t>
+  </si>
+  <si>
+    <t>Car_50L_10_1yr</t>
   </si>
 </sst>
 </file>
@@ -436,15 +436,15 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{6F1A2503-9150-498C-8314-EC557360F5D4}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{DD0AE97C-6A90-435A-BFB0-462DB7CBF186}">
   <dimension ref="A1:G4"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="1" max="1" width="12.453125" customWidth="1"/>
+    <col min="1" max="1" width="12.54296875" customWidth="1"/>
     <col min="2" max="2" width="11.54296875" customWidth="1"/>
-    <col min="4" max="4" width="15" customWidth="1"/>
-    <col min="5" max="5" width="12.81640625" customWidth="1"/>
-    <col min="6" max="6" width="11.1796875" customWidth="1"/>
+    <col min="4" max="4" width="16.54296875" customWidth="1"/>
+    <col min="5" max="5" width="15.6328125" customWidth="1"/>
+    <col min="6" max="6" width="12.54296875" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:7" x14ac:dyDescent="0.35">
@@ -458,16 +458,16 @@
         <v>2</v>
       </c>
       <c r="D1" t="s">
+        <v>6</v>
+      </c>
+      <c r="E1" t="s">
         <v>3</v>
       </c>
-      <c r="E1" t="s">
+      <c r="F1" t="s">
         <v>4</v>
       </c>
-      <c r="F1" t="s">
+      <c r="G1" t="s">
         <v>5</v>
-      </c>
-      <c r="G1" t="s">
-        <v>6</v>
       </c>
     </row>
     <row r="2" spans="1:7" x14ac:dyDescent="0.35">

</xml_diff>

<commit_message>
Modified CarLoanPage and CarLoanTest classes
</commit_message>
<xml_diff>
--- a/test-data/CarLoanTestData.xlsx
+++ b/test-data/CarLoanTestData.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Final Project\emi-calculator-automation\test-data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0C7D74B8-A45B-4E73-8F20-1AA01CF8A13E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{67A67B83-0AA7-44B9-9F13-3E1CF2E9658E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="12220" xr2:uid="{C06392C3-B2F8-4A4B-BB2F-76D7B47CBD86}"/>
   </bookViews>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="16" uniqueCount="11">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="14" uniqueCount="9">
   <si>
     <t>Loan Amount</t>
   </si>
@@ -60,12 +60,6 @@
   </si>
   <si>
     <t>Car_15L_9.5_1yr</t>
-  </si>
-  <si>
-    <t>Car_20L_8.5_1yr</t>
-  </si>
-  <si>
-    <t>Car_50L_10_1yr</t>
   </si>
   <si>
     <t>PASS</t>
@@ -76,7 +70,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
   <numFmts count="0"/>
-  <fonts count="8" x14ac:knownFonts="1">
+  <fonts count="9" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -101,14 +95,9 @@
     <font>
       <b/>
       <sz val="11"/>
-      <color indexed="9"/>
+      <color theme="1"/>
       <name val="Calibri"/>
-    </font>
-    <font>
-      <b/>
-      <sz val="11"/>
-      <color indexed="9"/>
-      <name val="Calibri"/>
+      <family val="2"/>
     </font>
     <font>
       <name val="Calibri"/>
@@ -128,8 +117,20 @@
       <b val="true"/>
       <color indexed="9"/>
     </font>
+    <font>
+      <name val="Calibri"/>
+      <sz val="11.0"/>
+      <b val="true"/>
+      <color indexed="9"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <sz val="11.0"/>
+      <b val="true"/>
+      <color indexed="9"/>
+    </font>
   </fonts>
-  <fills count="4">
+  <fills count="5">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -142,12 +143,18 @@
       </patternFill>
     </fill>
     <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="0"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
       <patternFill patternType="none">
         <fgColor indexed="17"/>
       </patternFill>
     </fill>
   </fills>
-  <borders count="1">
+  <borders count="3">
     <border>
       <left/>
       <right/>
@@ -155,20 +162,45 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top/>
+      <bottom style="thin">
+        <color theme="2" tint="-0.249977111117893"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="8">
+  <cellXfs count="10">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="3" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="4" fillId="2" borderId="0" xfId="0" applyFont="true" applyAlignment="true" applyFill="true">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="5" fillId="2" borderId="0" xfId="0" applyFont="true" applyAlignment="true" applyFill="true">
@@ -178,6 +210,9 @@
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="7" fillId="2" borderId="0" xfId="0" applyFont="true" applyAlignment="true" applyFill="true">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="2" borderId="0" xfId="0" applyFont="true" applyAlignment="true" applyFill="true">
       <alignment horizontal="center"/>
     </xf>
   </cellXfs>
@@ -514,7 +549,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{DD0AE97C-6A90-435A-BFB0-462DB7CBF186}">
-  <dimension ref="A1:G4"/>
+  <dimension ref="A1:G15"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" customWidth="true" width="12.54296875"/>
@@ -566,55 +601,18 @@
       <c r="F2" t="n" s="0">
         <v>131525.0</v>
       </c>
-      <c r="G2" s="5" t="s">
-        <v>10</v>
+      <c r="G2" s="9" t="s">
+        <v>8</v>
       </c>
     </row>
     <row r="3" spans="1:7" x14ac:dyDescent="0.35">
-      <c r="A3" s="0">
-        <v>2000000</v>
-      </c>
-      <c r="B3" s="0">
-        <v>8.5</v>
-      </c>
-      <c r="C3" s="0">
-        <v>2</v>
-      </c>
-      <c r="D3" t="s" s="0">
-        <v>8</v>
-      </c>
-      <c r="E3" s="0" t="n">
-        <v>90911.0</v>
-      </c>
-      <c r="F3" s="0" t="n">
-        <v>90911.0</v>
-      </c>
-      <c r="G3" s="6" t="s">
-        <v>10</v>
-      </c>
+      <c r="G3" s="3"/>
     </row>
     <row r="4" spans="1:7" x14ac:dyDescent="0.35">
-      <c r="A4" s="0">
-        <v>5000000</v>
-      </c>
-      <c r="B4" s="0">
-        <v>10</v>
-      </c>
-      <c r="C4" s="0">
-        <v>5</v>
-      </c>
-      <c r="D4" t="s" s="0">
-        <v>9</v>
-      </c>
-      <c r="E4" s="0" t="n">
-        <v>106235.0</v>
-      </c>
-      <c r="F4" s="0" t="n">
-        <v>106235.0</v>
-      </c>
-      <c r="G4" s="7" t="s">
-        <v>10</v>
-      </c>
+      <c r="G4" s="3"/>
+    </row>
+    <row r="15" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="F15" s="4"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>